<commit_message>
actualiza informe de precariedad
</commit_message>
<xml_diff>
--- a/resultados/indicadores_precariedad.xlsx
+++ b/resultados/indicadores_precariedad.xlsx
@@ -8,14 +8,18 @@
   <sheets>
     <sheet name="Resumen_General" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Por_Sexo_y_Edad" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Por_Tamano_Empresa" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Por_Aglomerado" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Por_Nivel_Educativo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Por_Tamano_Empresa" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Por_Aglomerado" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+  <si>
+    <t xml:space="preserve">casos_muestrales</t>
+  </si>
   <si>
     <t xml:space="preserve">poblacion_asalariada</t>
   </si>
@@ -23,6 +27,9 @@
     <t xml:space="preserve">precarios_ponderados</t>
   </si>
   <si>
+    <t xml:space="preserve">registrados_ponderados</t>
+  </si>
+  <si>
     <t xml:space="preserve">tasa_precariedad</t>
   </si>
   <si>
@@ -47,22 +54,133 @@
     <t xml:space="preserve">Varón</t>
   </si>
   <si>
+    <t xml:space="preserve">nivel_educativo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hasta secundario incompleto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secundario completo / superior incompleto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Superior universitario completo</t>
+  </si>
+  <si>
     <t xml:space="preserve">tamano_establec</t>
   </si>
   <si>
-    <t xml:space="preserve">Pequeño (hasta 10 pers.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mediano (11 a 50 pers.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grande (más de 50 pers.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NS/NR</t>
+    <t xml:space="preserve">Hasta 10 personas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 a 40 personas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">41 personas o más</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No sabe / no responde</t>
   </si>
   <si>
     <t xml:space="preserve">AGLOMERADO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nom_aglo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gran Tucumán - Tafí Viejo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concordia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gran San Juan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santiago del Estero - La Banda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Río Cuarto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formosa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gran Córdoba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gran Mendoza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Luis - El Chorrillo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrientes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gran Catamarca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jujuy - Palpalá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gran Resistencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partidos del GBA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gran La Plata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mar del Plata - Batán</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Rioja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gran Rosario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gran Paraná</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Nicolás - Villa Constitución</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santa Rosa - Toay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bahía Blanca - Cerri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gran Santa Fe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viedma - Carmen de Patagones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comodoro Rivadavia - Rada Tilly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciudad de Buenos Aires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rawson - Trelew</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neuquén - Plottier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Río Gallegos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ushuaia - Río Grande</t>
   </si>
 </sst>
 </file>
@@ -401,15 +519,27 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>15292</v>
+      </c>
+      <c r="B2" t="n">
         <v>9833243</v>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>3551642</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
+        <v>6281601</v>
+      </c>
+      <c r="E2" t="n">
         <v>0.361187250228638</v>
       </c>
     </row>
@@ -426,10 +556,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -440,106 +570,127 @@
       <c r="E1" t="s">
         <v>2</v>
       </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>1043964</v>
+        <v>1520</v>
       </c>
       <c r="D2" t="n">
-        <v>589427</v>
+        <v>1027066</v>
       </c>
       <c r="E2" t="n">
-        <v>0.564604718170358</v>
+        <v>575918</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.560740984513167</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" t="n">
+        <v>3822</v>
+      </c>
+      <c r="D3" t="n">
         <v>2448351</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>813898</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.332427009035878</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" t="n">
+        <v>1828</v>
+      </c>
+      <c r="D4" t="n">
         <v>1081117</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>350821</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0.324498643532569</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>1374643</v>
+        <v>2080</v>
       </c>
       <c r="D5" t="n">
-        <v>749832</v>
+        <v>1351359</v>
       </c>
       <c r="E5" t="n">
-        <v>0.545473988519201</v>
+        <v>726548</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.53764247694358</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
       <c r="C6" t="n">
+        <v>4090</v>
+      </c>
+      <c r="D6" t="n">
         <v>2714026</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>745639</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>0.274735393102351</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C7" t="n">
+        <v>1910</v>
+      </c>
+      <c r="D7" t="n">
         <v>1171142</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>302025</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>0.257889308042919</v>
       </c>
     </row>
@@ -556,7 +707,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -567,61 +718,59 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B2" t="n">
-        <v>4075658</v>
+        <v>4132</v>
       </c>
       <c r="C2" t="n">
-        <v>1941292</v>
+        <v>2524313</v>
       </c>
       <c r="D2" t="n">
-        <v>0.476313763323615</v>
+        <v>1465513</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.580559146191459</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B3" t="n">
-        <v>2847722</v>
+        <v>7204</v>
       </c>
       <c r="C3" t="n">
-        <v>255527</v>
+        <v>4537176</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0897303177768055</v>
+        <v>1669130</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.367878609954738</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B4" t="n">
-        <v>2072396</v>
+        <v>3956</v>
       </c>
       <c r="C4" t="n">
-        <v>712688</v>
+        <v>2771754</v>
       </c>
       <c r="D4" t="n">
-        <v>0.34389566472817</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="n">
-        <v>837467</v>
-      </c>
-      <c r="C5" t="n">
-        <v>642135</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.766758570785476</v>
+        <v>416999</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.15044589094126</v>
       </c>
     </row>
   </sheetData>
@@ -637,7 +786,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -648,453 +797,747 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="n">
+        <v>4094</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2493086</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1599697</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.641653356522799</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2936</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1582572</v>
+      </c>
+      <c r="D3" t="n">
+        <v>341595</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.215847999332732</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="n">
+        <v>4203</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2847722</v>
+      </c>
+      <c r="D4" t="n">
+        <v>255527</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0897303177768055</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2650</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2072396</v>
+      </c>
+      <c r="D5" t="n">
+        <v>712688</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.34389566472817</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B2" t="n">
-        <v>346578</v>
+        <v>29</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
       </c>
       <c r="C2" t="n">
-        <v>124288</v>
+        <v>723</v>
       </c>
       <c r="D2" t="n">
-        <v>0.358614799554501</v>
+        <v>289320</v>
+      </c>
+      <c r="E2" t="n">
+        <v>148837</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.514437301258122</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B3" t="n">
-        <v>107750</v>
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
       </c>
       <c r="C3" t="n">
-        <v>31384</v>
+        <v>397</v>
       </c>
       <c r="D3" t="n">
-        <v>0.291266821345708</v>
+        <v>49299</v>
+      </c>
+      <c r="E3" t="n">
+        <v>24297</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.492849753544697</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B4" t="n">
-        <v>460986</v>
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
       </c>
       <c r="C4" t="n">
-        <v>142602</v>
+        <v>471</v>
       </c>
       <c r="D4" t="n">
-        <v>0.309341281513972</v>
+        <v>164963</v>
+      </c>
+      <c r="E4" t="n">
+        <v>80300</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.486775822457157</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B5" t="n">
-        <v>155893</v>
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
       </c>
       <c r="C5" t="n">
-        <v>45315</v>
+        <v>433</v>
       </c>
       <c r="D5" t="n">
-        <v>0.290680145997575</v>
+        <v>123267</v>
+      </c>
+      <c r="E5" t="n">
+        <v>55867</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.453219434236251</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B6" t="n">
-        <v>83424</v>
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
       </c>
       <c r="C6" t="n">
-        <v>25753</v>
+        <v>603</v>
       </c>
       <c r="D6" t="n">
-        <v>0.308700134253932</v>
+        <v>194559</v>
+      </c>
+      <c r="E6" t="n">
+        <v>86910</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.446702542673431</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B7" t="n">
-        <v>118229</v>
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
       </c>
       <c r="C7" t="n">
-        <v>45015</v>
+        <v>333</v>
       </c>
       <c r="D7" t="n">
-        <v>0.380744149066642</v>
+        <v>58070</v>
+      </c>
+      <c r="E7" t="n">
+        <v>25666</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.441983812639917</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>8</v>
-      </c>
-      <c r="B8" t="n">
-        <v>128416</v>
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
       </c>
       <c r="C8" t="n">
-        <v>49185</v>
+        <v>335</v>
       </c>
       <c r="D8" t="n">
-        <v>0.383013020184401</v>
+        <v>71419</v>
+      </c>
+      <c r="E8" t="n">
+        <v>30925</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.433008023075092</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B9" t="n">
-        <v>80796</v>
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
       </c>
       <c r="C9" t="n">
-        <v>19235</v>
+        <v>706</v>
       </c>
       <c r="D9" t="n">
-        <v>0.238068716273083</v>
+        <v>549604</v>
+      </c>
+      <c r="E9" t="n">
+        <v>237715</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.432520505673176</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
         <v>10</v>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" t="n">
+        <v>602</v>
+      </c>
+      <c r="D10" t="n">
         <v>343283</v>
       </c>
-      <c r="C10" t="n">
+      <c r="E10" t="n">
         <v>146713</v>
       </c>
-      <c r="D10" t="n">
+      <c r="F10" t="n">
         <v>0.427382072517427</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>12</v>
-      </c>
-      <c r="B11" t="n">
-        <v>117764</v>
+        <v>26</v>
+      </c>
+      <c r="B11" t="s">
+        <v>32</v>
       </c>
       <c r="C11" t="n">
-        <v>49838</v>
+        <v>421</v>
       </c>
       <c r="D11" t="n">
-        <v>0.423202336877144</v>
+        <v>85740</v>
+      </c>
+      <c r="E11" t="n">
+        <v>36561</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.426417074877537</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>13</v>
-      </c>
-      <c r="B12" t="n">
-        <v>549604</v>
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>33</v>
       </c>
       <c r="C12" t="n">
-        <v>237715</v>
+        <v>308</v>
       </c>
       <c r="D12" t="n">
-        <v>0.432520505673176</v>
+        <v>117764</v>
+      </c>
+      <c r="E12" t="n">
+        <v>49838</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.423202336877144</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>14</v>
-      </c>
-      <c r="B13" t="n">
-        <v>49299</v>
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>34</v>
       </c>
       <c r="C13" t="n">
-        <v>24297</v>
+        <v>517</v>
       </c>
       <c r="D13" t="n">
-        <v>0.492849753544697</v>
+        <v>78592</v>
+      </c>
+      <c r="E13" t="n">
+        <v>32786</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.417167141693811</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>15</v>
-      </c>
-      <c r="B14" t="n">
-        <v>71419</v>
+        <v>19</v>
+      </c>
+      <c r="B14" t="s">
+        <v>35</v>
       </c>
       <c r="C14" t="n">
-        <v>30925</v>
+        <v>499</v>
       </c>
       <c r="D14" t="n">
-        <v>0.433008023075092</v>
+        <v>117983</v>
+      </c>
+      <c r="E14" t="n">
+        <v>46955</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.397981065068696</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>17</v>
-      </c>
-      <c r="B15" t="n">
-        <v>122020</v>
+        <v>8</v>
+      </c>
+      <c r="B15" t="s">
+        <v>36</v>
       </c>
       <c r="C15" t="n">
-        <v>24711</v>
+        <v>398</v>
       </c>
       <c r="D15" t="n">
-        <v>0.202515980986723</v>
+        <v>128416</v>
+      </c>
+      <c r="E15" t="n">
+        <v>49185</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.383013020184401</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>18</v>
-      </c>
-      <c r="B16" t="n">
-        <v>123267</v>
+        <v>7</v>
+      </c>
+      <c r="B16" t="s">
+        <v>37</v>
       </c>
       <c r="C16" t="n">
-        <v>55867</v>
+        <v>376</v>
       </c>
       <c r="D16" t="n">
-        <v>0.453219434236251</v>
+        <v>118229</v>
+      </c>
+      <c r="E16" t="n">
+        <v>45015</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.380744149066642</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>19</v>
-      </c>
-      <c r="B17" t="n">
-        <v>117983</v>
+        <v>33</v>
+      </c>
+      <c r="B17" t="s">
+        <v>38</v>
       </c>
       <c r="C17" t="n">
-        <v>46955</v>
+        <v>2032</v>
       </c>
       <c r="D17" t="n">
-        <v>0.397981065068696</v>
+        <v>4219215</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1603341</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.380009314528887</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>20</v>
-      </c>
-      <c r="B18" t="n">
-        <v>48340</v>
+        <v>2</v>
+      </c>
+      <c r="B18" t="s">
+        <v>39</v>
       </c>
       <c r="C18" t="n">
-        <v>7369</v>
+        <v>363</v>
       </c>
       <c r="D18" t="n">
-        <v>0.152441042614812</v>
+        <v>346578</v>
+      </c>
+      <c r="E18" t="n">
+        <v>124288</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.358614799554501</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>22</v>
-      </c>
-      <c r="B19" t="n">
-        <v>78592</v>
+        <v>34</v>
+      </c>
+      <c r="B19" t="s">
+        <v>40</v>
       </c>
       <c r="C19" t="n">
-        <v>32786</v>
+        <v>279</v>
       </c>
       <c r="D19" t="n">
-        <v>0.417167141693811</v>
+        <v>203735</v>
+      </c>
+      <c r="E19" t="n">
+        <v>66561</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.326703806415196</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>23</v>
-      </c>
-      <c r="B20" t="n">
-        <v>194559</v>
+        <v>25</v>
+      </c>
+      <c r="B20" t="s">
+        <v>41</v>
       </c>
       <c r="C20" t="n">
-        <v>86910</v>
+        <v>476</v>
       </c>
       <c r="D20" t="n">
-        <v>0.446702542673431</v>
+        <v>86912</v>
+      </c>
+      <c r="E20" t="n">
+        <v>27603</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.317597109720177</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>25</v>
-      </c>
-      <c r="B21" t="n">
-        <v>86912</v>
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>42</v>
       </c>
       <c r="C21" t="n">
-        <v>27603</v>
+        <v>539</v>
       </c>
       <c r="D21" t="n">
-        <v>0.317597109720177</v>
+        <v>460986</v>
+      </c>
+      <c r="E21" t="n">
+        <v>142602</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.309341281513972</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>26</v>
-      </c>
-      <c r="B22" t="n">
-        <v>85740</v>
+        <v>6</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
       </c>
       <c r="C22" t="n">
-        <v>36561</v>
+        <v>396</v>
       </c>
       <c r="D22" t="n">
-        <v>0.426417074877537</v>
+        <v>83424</v>
+      </c>
+      <c r="E22" t="n">
+        <v>25753</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.308700134253932</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>27</v>
-      </c>
-      <c r="B23" t="n">
-        <v>164963</v>
+        <v>38</v>
+      </c>
+      <c r="B23" t="s">
+        <v>44</v>
       </c>
       <c r="C23" t="n">
-        <v>80300</v>
+        <v>433</v>
       </c>
       <c r="D23" t="n">
-        <v>0.486775822457157</v>
+        <v>56094</v>
+      </c>
+      <c r="E23" t="n">
+        <v>17287</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.308179127892466</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>29</v>
-      </c>
-      <c r="B24" t="n">
-        <v>289320</v>
+        <v>30</v>
+      </c>
+      <c r="B24" t="s">
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>148837</v>
+        <v>294</v>
       </c>
       <c r="D24" t="n">
-        <v>0.514437301258122</v>
+        <v>45580</v>
+      </c>
+      <c r="E24" t="n">
+        <v>13677</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.300065818341378</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>30</v>
-      </c>
-      <c r="B25" t="n">
-        <v>45580</v>
+        <v>3</v>
+      </c>
+      <c r="B25" t="s">
+        <v>46</v>
       </c>
       <c r="C25" t="n">
-        <v>13677</v>
+        <v>338</v>
       </c>
       <c r="D25" t="n">
-        <v>0.300065818341378</v>
+        <v>107750</v>
+      </c>
+      <c r="E25" t="n">
+        <v>31384</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.291266821345708</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>31</v>
-      </c>
-      <c r="B26" t="n">
-        <v>68343</v>
+        <v>5</v>
+      </c>
+      <c r="B26" t="s">
+        <v>47</v>
       </c>
       <c r="C26" t="n">
-        <v>9453</v>
+        <v>400</v>
       </c>
       <c r="D26" t="n">
-        <v>0.138317018568105</v>
+        <v>155893</v>
+      </c>
+      <c r="E26" t="n">
+        <v>45315</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.290680145997575</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>32</v>
-      </c>
-      <c r="B27" t="n">
-        <v>1180901</v>
+        <v>93</v>
+      </c>
+      <c r="B27" t="s">
+        <v>48</v>
       </c>
       <c r="C27" t="n">
-        <v>277207</v>
+        <v>284</v>
       </c>
       <c r="D27" t="n">
-        <v>0.234741947038744</v>
+        <v>26102</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7056</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.270324113094782</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>33</v>
-      </c>
-      <c r="B28" t="n">
-        <v>4219215</v>
+        <v>9</v>
+      </c>
+      <c r="B28" t="s">
+        <v>49</v>
       </c>
       <c r="C28" t="n">
-        <v>1603341</v>
+        <v>248</v>
       </c>
       <c r="D28" t="n">
-        <v>0.380009314528887</v>
+        <v>80796</v>
+      </c>
+      <c r="E28" t="n">
+        <v>19235</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.238068716273083</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>34</v>
-      </c>
-      <c r="B29" t="n">
-        <v>203735</v>
+        <v>32</v>
+      </c>
+      <c r="B29" t="s">
+        <v>50</v>
       </c>
       <c r="C29" t="n">
-        <v>66561</v>
+        <v>642</v>
       </c>
       <c r="D29" t="n">
-        <v>0.326703806415196</v>
+        <v>1180901</v>
+      </c>
+      <c r="E29" t="n">
+        <v>277207</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.234741947038744</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>36</v>
-      </c>
-      <c r="B30" t="n">
-        <v>58070</v>
+        <v>91</v>
+      </c>
+      <c r="B30" t="s">
+        <v>51</v>
       </c>
       <c r="C30" t="n">
-        <v>25666</v>
+        <v>303</v>
       </c>
       <c r="D30" t="n">
-        <v>0.441983812639917</v>
+        <v>50066</v>
+      </c>
+      <c r="E30" t="n">
+        <v>11230</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.224303918827148</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>38</v>
-      </c>
-      <c r="B31" t="n">
-        <v>56094</v>
+        <v>17</v>
+      </c>
+      <c r="B31" t="s">
+        <v>52</v>
       </c>
       <c r="C31" t="n">
-        <v>17287</v>
+        <v>453</v>
       </c>
       <c r="D31" t="n">
-        <v>0.308179127892466</v>
+        <v>122020</v>
+      </c>
+      <c r="E31" t="n">
+        <v>24711</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.202515980986723</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>91</v>
-      </c>
-      <c r="B32" t="n">
-        <v>50066</v>
+        <v>20</v>
+      </c>
+      <c r="B32" t="s">
+        <v>53</v>
       </c>
       <c r="C32" t="n">
-        <v>11230</v>
+        <v>279</v>
       </c>
       <c r="D32" t="n">
-        <v>0.224303918827148</v>
+        <v>48340</v>
+      </c>
+      <c r="E32" t="n">
+        <v>7369</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.152441042614812</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>93</v>
-      </c>
-      <c r="B33" t="n">
-        <v>26102</v>
+        <v>31</v>
+      </c>
+      <c r="B33" t="s">
+        <v>54</v>
       </c>
       <c r="C33" t="n">
-        <v>7056</v>
+        <v>411</v>
       </c>
       <c r="D33" t="n">
-        <v>0.270324113094782</v>
+        <v>68343</v>
+      </c>
+      <c r="E33" t="n">
+        <v>9453</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.138317018568105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>